<commit_message>
test(e2e): add comprehensive article update test suite with security payload coverage
- add full Article Update specification (happy, negative, edge scenarios)
- introduce dedicated article-update fixture and editor/detail helper methods
- add reusable SQLi and XSS payload factories plus escaped-content UI assertions
- unify article create/update API route helper via ARTICLES.SAVE
- refactor test article id generation to CompositeIdFactory.fromExecutionInfo
- update article creation/read specs and test inventory coverage docs

Refs: #10
</commit_message>
<xml_diff>
--- a/docs/tests-inventories/0002_article-inventory.xlsx
+++ b/docs/tests-inventories/0002_article-inventory.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="190">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -428,142 +428,142 @@
     <t xml:space="preserve">Article-update.spec.ts</t>
   </si>
   <si>
+    <t xml:space="preserve">ARTICLE-U-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article title successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article description successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article body successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article tags successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article tags with empty value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current title when title is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current description when description is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current body when body is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trying to access another user's article editor redirects to home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article tags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unauthenticated user trying to update an article is redirected to the home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">handle concurrent updates on the same article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cancel update without saving changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prefill form with existing article data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disable form when update request is pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent duplicate submit on double click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-D-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete article successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article-Delete.spec.ts</t>
+  </si>
+  <si>
     <t xml:space="preserve">Missing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article title successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article description successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article body successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article tags successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article tags with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep current title when title is empty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article description with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article body with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article another user article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-107</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-108</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-109</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article body</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article tags</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-112</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent unauthenticated user from updating article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">handle concurrent updates on the same article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cancel update without saving changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prefill form with existing article data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disable form when update request is pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent duplicate submit on double click</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-D-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delete article successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article-Delete.spec.ts</t>
   </si>
   <si>
     <t xml:space="preserve">ARTICLE-D-100</t>
@@ -800,19 +800,19 @@
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D3:D27,"*Happy*",Update!G3:G27,"*done*")/COUNTIF(Update!D3:D27,"*happy*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D2:D27,"*Negative*",Update!G2:G27,"*done*")/COUNTIF(Update!D2:D27,"*Negative*")</f>
-        <v>0</v>
+        <v>0.923076923076923</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D2:D27,"*Edge*",Update!G2:G27,"*done*")/COUNTIF(Update!D2:D27,"*Edge*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">AVERAGE(B4:D4)</f>
-        <v>0</v>
+        <v>0.974358974358974</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -842,19 +842,19 @@
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">AVERAGE(B2:B5)</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="C6" s="4" t="n">
         <f aca="false">AVERAGE(C2:C5)</f>
-        <v>0.375</v>
+        <v>0.605769230769231</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">AVERAGE(D2:D5)</f>
-        <v>0.152777777777778</v>
+        <v>0.402777777777778</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">AVERAGE(E2:E5)</f>
-        <v>0.342592592592592</v>
+        <v>0.586182336182336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3316,7 +3316,7 @@
         <v>133</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -3325,10 +3325,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>21</v>
@@ -3340,7 +3340,7 @@
         <v>133</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3348,10 +3348,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>21</v>
@@ -3363,7 +3363,7 @@
         <v>133</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3371,10 +3371,10 @@
         <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>21</v>
@@ -3386,7 +3386,7 @@
         <v>133</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3394,10 +3394,10 @@
         <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>21</v>
@@ -3409,7 +3409,7 @@
         <v>133</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3417,10 +3417,10 @@
         <v>18</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>21</v>
@@ -3432,7 +3432,7 @@
         <v>133</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3440,10 +3440,10 @@
         <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>35</v>
@@ -3455,7 +3455,7 @@
         <v>133</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3463,10 +3463,10 @@
         <v>18</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>35</v>
@@ -3478,7 +3478,7 @@
         <v>133</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,10 +3486,10 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>35</v>
@@ -3501,7 +3501,7 @@
         <v>133</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3509,10 +3509,10 @@
         <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>35</v>
@@ -3524,7 +3524,7 @@
         <v>133</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3532,7 +3532,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>48</v>
@@ -3547,7 +3547,7 @@
         <v>133</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3555,7 +3555,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>51</v>
@@ -3570,7 +3570,7 @@
         <v>133</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,7 +3578,7 @@
         <v>18</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>53</v>
@@ -3593,7 +3593,7 @@
         <v>133</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3601,7 +3601,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>55</v>
@@ -3616,7 +3616,7 @@
         <v>133</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,10 +3624,10 @@
         <v>18</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>35</v>
@@ -3639,7 +3639,7 @@
         <v>133</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3647,10 +3647,10 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>35</v>
@@ -3662,7 +3662,7 @@
         <v>133</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,10 +3670,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>35</v>
@@ -3685,7 +3685,7 @@
         <v>133</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3693,10 +3693,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>35</v>
@@ -3708,7 +3708,7 @@
         <v>133</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,10 +3716,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>35</v>
@@ -3731,7 +3731,10 @@
         <v>133</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>134</v>
+        <v>36</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3739,10 +3742,10 @@
         <v>18</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>73</v>
@@ -3754,7 +3757,7 @@
         <v>133</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,10 +3765,10 @@
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>73</v>
@@ -3777,7 +3780,7 @@
         <v>133</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3785,10 +3788,10 @@
         <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>73</v>
@@ -3800,7 +3803,7 @@
         <v>133</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3808,10 +3811,10 @@
         <v>18</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>73</v>
@@ -3823,7 +3826,7 @@
         <v>133</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3831,10 +3834,10 @@
         <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>73</v>
@@ -3846,7 +3849,7 @@
         <v>133</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -3909,10 +3912,10 @@
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>178</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>21</v>
@@ -3921,10 +3924,10 @@
         <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,10 +3947,10 @@
         <v>27</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3967,10 +3970,10 @@
         <v>27</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3990,10 +3993,10 @@
         <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4013,10 +4016,10 @@
         <v>27</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,10 +4039,10 @@
         <v>27</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[#10] Add E2E tests for article update (#16)
* test(e2e): add comprehensive article update test suite with security payload coverage

- add full Article Update specification (happy, negative, edge scenarios)
- introduce dedicated article-update fixture and editor/detail helper methods
- add reusable SQLi and XSS payload factories plus escaped-content UI assertions
- unify article create/update API route helper via ARTICLES.SAVE
- refactor test article id generation to CompositeIdFactory.fromExecutionInfo
- update article creation/read specs and test inventory coverage docs

Refs: #10

* test(article-update): replace skip with fixme and add issue annotation for unauthenticated edit scenario

Refs: #10

* chore(config): retain trace only on first failure

Refs: #10

* refactor(e2e): move test tree to tests/features, rename specs to *.e2e.spec.ts, and align config

Refs: #10

---------

Co-authored-by: idembele70 <idembele70@gmail>
</commit_message>
<xml_diff>
--- a/docs/tests-inventories/0002_article-inventory.xlsx
+++ b/docs/tests-inventories/0002_article-inventory.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="190">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -428,142 +428,142 @@
     <t xml:space="preserve">Article-update.spec.ts</t>
   </si>
   <si>
+    <t xml:space="preserve">ARTICLE-U-002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article title successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article description successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article body successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article tags successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update article tags with empty value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current title when title is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current description when description is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep current body when body is empty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trying to access another user's article editor redirects to home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-109</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent HTML injection in article tags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unauthenticated user trying to update an article is redirected to the home page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">handle concurrent updates on the same article</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cancel update without saving changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-202</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prefill form with existing article data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disable form when update request is pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-U-204</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prevent duplicate submit on double click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARTICLE-D-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete article successfully</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Article-Delete.spec.ts</t>
+  </si>
+  <si>
     <t xml:space="preserve">Missing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article title successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article description successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article body successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article tags successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update article tags with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep current title when title is empty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article description with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article body with empty value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-103</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modify article another user article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-107</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-108</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-109</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article body</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent HTML injection in article tags</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-112</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent unauthenticated user from updating article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">handle concurrent updates on the same article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-201</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cancel update without saving changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-202</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prefill form with existing article data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-203</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disable form when update request is pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-U-204</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevent duplicate submit on double click</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ARTICLE-D-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delete article successfully</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Article-Delete.spec.ts</t>
   </si>
   <si>
     <t xml:space="preserve">ARTICLE-D-100</t>
@@ -800,19 +800,19 @@
       </c>
       <c r="B4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D3:D27,"*Happy*",Update!G3:G27,"*done*")/COUNTIF(Update!D3:D27,"*happy*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D2:D27,"*Negative*",Update!G2:G27,"*done*")/COUNTIF(Update!D2:D27,"*Negative*")</f>
-        <v>0</v>
+        <v>0.923076923076923</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIFS(Update!D2:D27,"*Edge*",Update!G2:G27,"*done*")/COUNTIF(Update!D2:D27,"*Edge*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">AVERAGE(B4:D4)</f>
-        <v>0</v>
+        <v>0.974358974358974</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -842,19 +842,19 @@
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">AVERAGE(B2:B5)</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="C6" s="4" t="n">
         <f aca="false">AVERAGE(C2:C5)</f>
-        <v>0.375</v>
+        <v>0.605769230769231</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">AVERAGE(D2:D5)</f>
-        <v>0.152777777777778</v>
+        <v>0.402777777777778</v>
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">AVERAGE(E2:E5)</f>
-        <v>0.342592592592592</v>
+        <v>0.586182336182336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3316,7 +3316,7 @@
         <v>133</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -3325,10 +3325,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>21</v>
@@ -3340,7 +3340,7 @@
         <v>133</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3348,10 +3348,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>21</v>
@@ -3363,7 +3363,7 @@
         <v>133</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3371,10 +3371,10 @@
         <v>18</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>21</v>
@@ -3386,7 +3386,7 @@
         <v>133</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3394,10 +3394,10 @@
         <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>21</v>
@@ -3409,7 +3409,7 @@
         <v>133</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3417,10 +3417,10 @@
         <v>18</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>21</v>
@@ -3432,7 +3432,7 @@
         <v>133</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3440,10 +3440,10 @@
         <v>18</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>35</v>
@@ -3455,7 +3455,7 @@
         <v>133</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3463,10 +3463,10 @@
         <v>18</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>35</v>
@@ -3478,7 +3478,7 @@
         <v>133</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,10 +3486,10 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>35</v>
@@ -3501,7 +3501,7 @@
         <v>133</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3509,10 +3509,10 @@
         <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>35</v>
@@ -3524,7 +3524,7 @@
         <v>133</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3532,7 +3532,7 @@
         <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>48</v>
@@ -3547,7 +3547,7 @@
         <v>133</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3555,7 +3555,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>51</v>
@@ -3570,7 +3570,7 @@
         <v>133</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3578,7 +3578,7 @@
         <v>18</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>53</v>
@@ -3593,7 +3593,7 @@
         <v>133</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3601,7 +3601,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>55</v>
@@ -3616,7 +3616,7 @@
         <v>133</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,10 +3624,10 @@
         <v>18</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>35</v>
@@ -3639,7 +3639,7 @@
         <v>133</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3647,10 +3647,10 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>35</v>
@@ -3662,7 +3662,7 @@
         <v>133</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,10 +3670,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>35</v>
@@ -3685,7 +3685,7 @@
         <v>133</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3693,10 +3693,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>35</v>
@@ -3708,7 +3708,7 @@
         <v>133</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,10 +3716,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>35</v>
@@ -3731,7 +3731,10 @@
         <v>133</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>134</v>
+        <v>36</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3739,10 +3742,10 @@
         <v>18</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>73</v>
@@ -3754,7 +3757,7 @@
         <v>133</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3762,10 +3765,10 @@
         <v>18</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>73</v>
@@ -3777,7 +3780,7 @@
         <v>133</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3785,10 +3788,10 @@
         <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>73</v>
@@ -3800,7 +3803,7 @@
         <v>133</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3808,10 +3811,10 @@
         <v>18</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>73</v>
@@ -3823,7 +3826,7 @@
         <v>133</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3831,10 +3834,10 @@
         <v>18</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>73</v>
@@ -3846,7 +3849,7 @@
         <v>133</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>134</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -3909,10 +3912,10 @@
         <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>178</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>21</v>
@@ -3921,10 +3924,10 @@
         <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,10 +3947,10 @@
         <v>27</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3967,10 +3970,10 @@
         <v>27</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3990,10 +3993,10 @@
         <v>22</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4013,10 +4016,10 @@
         <v>27</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="18.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,10 +4039,10 @@
         <v>27</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>